<commit_message>
Fix malformed 2026 schedule source entries
</commit_message>
<xml_diff>
--- a/output/all_teachers_orar.xlsx
+++ b/output/all_teachers_orar.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="main" sheetId="1" r:id="R025498663fd54f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="main" sheetId="1" r:id="R2f3175dbd9334e87"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,7 +571,7 @@
     <x:t>Fund. progr. (lab) 251/4 IA2604-II</x:t>
   </x:si>
   <x:si>
-    <x:t>) 143/4 DJ2502</x:t>
+    <x:t>Progr. C++ (lab) 143/4 DJ2502</x:t>
   </x:si>
   <x:si>
     <x:t>Geom. dif. (sem) 214/4 M2501</x:t>
@@ -583,7 +583,7 @@
     <x:t>DJ3DU (curs) 423/4</x:t>
   </x:si>
   <x:si>
-    <x:t>) 350/4 DJ2502</x:t>
+    <x:t>DCMIMJ (lab) 350/4 DJ2502</x:t>
   </x:si>
   <x:si>
     <x:t>Sist. de oper. (lab) 145a/4 DU-IA2601</x:t>

</xml_diff>

<commit_message>
Add schedule import workflow and republish outputs
</commit_message>
<xml_diff>
--- a/output/all_teachers_orar.xlsx
+++ b/output/all_teachers_orar.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="main" sheetId="1" r:id="R2f3175dbd9334e87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="main" sheetId="1" r:id="R6368b1b1aa464381"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1110,7 +1110,7 @@
         <x:v>Cucu I.</x:v>
       </x:c>
       <x:c s="3" t="str">
-        <x:v>Curmanscii A.</x:v>
+        <x:v>Curmanschii Anton</x:v>
       </x:c>
       <x:c s="3" t="str">
         <x:v>Damian F.</x:v>

</xml_diff>